<commit_message>
updating version number in metadata
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-PL.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-PL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/schirico/IOTC/IOTC_reference_forms/form_reporting_templates/ros/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{699AC24F-3C11-4643-9C8D-35FF3161F88A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{439D3E0E-A178-EE43-B975-D79DB46C2DB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="24660" windowHeight="16840" tabRatio="803" firstSheet="10" activeTab="14" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="24660" windowHeight="16740" tabRatio="803" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="35" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="191">
   <si>
     <t>LATITUDE</t>
   </si>
@@ -278,9 +278,6 @@
   </si>
   <si>
     <t>Version</t>
-  </si>
-  <si>
-    <t>2.0.0</t>
   </si>
   <si>
     <t>Submission information</t>
@@ -1218,6 +1215,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1292,19 +1292,7 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1346,6 +1334,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1718,7 +1715,7 @@
     <row r="1" spans="2:8" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B2" s="61" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -1742,14 +1739,14 @@
         <v>74</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E4" s="10"/>
       <c r="F4" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="G4" s="11" t="s">
-        <v>76</v>
+      <c r="G4" s="11">
+        <v>4</v>
       </c>
       <c r="H4" s="12"/>
     </row>
@@ -1765,7 +1762,7 @@
     <row r="6" spans="2:8" ht="19" x14ac:dyDescent="0.25">
       <c r="B6" s="13"/>
       <c r="C6" s="16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
@@ -1785,12 +1782,12 @@
     <row r="8" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B8" s="13"/>
       <c r="C8" s="67" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D8" s="67"/>
       <c r="E8" s="14"/>
       <c r="F8" s="67" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G8" s="67"/>
       <c r="H8" s="15"/>
@@ -1798,12 +1795,12 @@
     <row r="9" spans="2:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="13"/>
       <c r="C9" s="17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D9" s="18"/>
       <c r="E9" s="14"/>
       <c r="F9" s="17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G9" s="18"/>
       <c r="H9" s="15"/>
@@ -1811,12 +1808,12 @@
     <row r="10" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B10" s="13"/>
       <c r="C10" s="19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D10" s="18"/>
       <c r="E10" s="14"/>
       <c r="F10" s="14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G10" s="18"/>
       <c r="H10" s="15"/>
@@ -1833,7 +1830,7 @@
     <row r="12" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B12" s="13"/>
       <c r="C12" s="19" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D12" s="21"/>
       <c r="E12" s="14"/>
@@ -1873,7 +1870,7 @@
     <row r="16" spans="2:8" ht="19" x14ac:dyDescent="0.25">
       <c r="B16" s="13"/>
       <c r="C16" s="16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D16" s="14"/>
       <c r="E16" s="14"/>
@@ -1893,7 +1890,7 @@
     <row r="18" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B18" s="13"/>
       <c r="C18" s="19" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D18" s="23"/>
       <c r="E18" s="14"/>
@@ -1904,7 +1901,7 @@
     <row r="19" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B19" s="13"/>
       <c r="C19" s="24" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D19" s="23"/>
       <c r="E19" s="14"/>
@@ -1926,7 +1923,7 @@
     <row r="21" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B21" s="13"/>
       <c r="C21" s="60" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D21" s="23"/>
       <c r="E21" s="14"/>
@@ -1995,7 +1992,7 @@
       <c r="D28" s="30"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="L0Y8Wko3eP5Yq8pEijOk1nzB+1M0apYi9uBJGWynVndNbEc8Y6vufqElebv2iCkLeSg4rtJpaBGk29mbM06vBw==" saltValue="fXrIfiTxdhPO9Ilm54xaVw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="bIHVKW/9SYUEMp5j00ENytYaPcpDZDdTvNpX4KPu4yNeLRi4urPwZ63Qp8YGQoDSk/Z/SXtQUbNTdTTgzVQUtg==" saltValue="8yroYgwpWbBbiCqQQUDBsg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="4">
     <mergeCell ref="B2:H3"/>
     <mergeCell ref="C8:D8"/>
@@ -2058,22 +2055,22 @@
         <v>67</v>
       </c>
       <c r="B1" s="127" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C1" s="127" t="s">
         <v>68</v>
       </c>
-      <c r="D1" s="89" t="s">
-        <v>143</v>
+      <c r="D1" s="90" t="s">
+        <v>142</v>
       </c>
       <c r="E1" s="71" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F1" s="71"/>
       <c r="G1" s="71"/>
       <c r="H1" s="71"/>
       <c r="I1" s="72" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J1" s="72"/>
       <c r="K1" s="72"/>
@@ -2083,7 +2080,7 @@
       </c>
       <c r="N1" s="72"/>
       <c r="O1" s="72"/>
-      <c r="P1" s="80" t="s">
+      <c r="P1" s="81" t="s">
         <v>37</v>
       </c>
       <c r="Q1" s="73" t="s">
@@ -2091,12 +2088,12 @@
       </c>
       <c r="R1" s="75"/>
       <c r="S1" s="72" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="T1" s="72"/>
       <c r="U1" s="72"/>
       <c r="V1" s="72" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="W1" s="72"/>
       <c r="X1" s="72"/>
@@ -2109,7 +2106,7 @@
       <c r="A2" s="128"/>
       <c r="B2" s="128"/>
       <c r="C2" s="128"/>
-      <c r="D2" s="91"/>
+      <c r="D2" s="92"/>
       <c r="E2" s="41" t="s">
         <v>54</v>
       </c>
@@ -2117,7 +2114,7 @@
         <v>36</v>
       </c>
       <c r="G2" s="41" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H2" s="31" t="s">
         <v>44</v>
@@ -2129,21 +2126,21 @@
         <v>36</v>
       </c>
       <c r="K2" s="35" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="L2" s="32" t="s">
         <v>44</v>
       </c>
       <c r="M2" s="35" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="N2" s="32" t="s">
         <v>35</v>
       </c>
       <c r="O2" s="35" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
-      <c r="P2" s="81"/>
+      <c r="P2" s="82"/>
       <c r="Q2" s="34" t="s">
         <v>56</v>
       </c>
@@ -2157,7 +2154,7 @@
         <v>38</v>
       </c>
       <c r="U2" s="58" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="V2" s="32" t="s">
         <v>39</v>
@@ -2169,10 +2166,10 @@
         <v>54</v>
       </c>
       <c r="Y2" s="32" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="Z2" s="32" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AA2" s="32" t="s">
         <v>69</v>
@@ -8184,17 +8181,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="HslEuID6IjZtZdKCUOojygIr7JEfDdTW3xXhdfKVBBZXMUg8BpmKsrISBeACUnUATtRkRZOGAip7oxU+3PrcFA==" saltValue="p7kZbF4A7qKywshOKE8NhA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="11">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="P1:P2"/>
-    <mergeCell ref="Q1:R1"/>
     <mergeCell ref="S1:U1"/>
     <mergeCell ref="V1:AB1"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="E1:H1"/>
     <mergeCell ref="I1:L1"/>
     <mergeCell ref="M1:O1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="P1:P2"/>
+    <mergeCell ref="Q1:R1"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2 D1:D2 E2 G2 I2 K2 P1:P2" xr:uid="{5E4B3162-4EBB-4AB5-B30D-164A47D38785}">
@@ -8246,19 +8243,19 @@
         <v>67</v>
       </c>
       <c r="B1" s="127" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C1" s="127" t="s">
         <v>68</v>
       </c>
-      <c r="D1" s="80" t="s">
-        <v>148</v>
+      <c r="D1" s="81" t="s">
+        <v>147</v>
       </c>
       <c r="E1" s="78" t="s">
         <v>41</v>
       </c>
-      <c r="F1" s="80" t="s">
-        <v>149</v>
+      <c r="F1" s="81" t="s">
+        <v>148</v>
       </c>
       <c r="G1" s="78" t="s">
         <v>42</v>
@@ -8266,18 +8263,18 @@
       <c r="H1" s="78" t="s">
         <v>43</v>
       </c>
-      <c r="I1" s="95" t="s">
-        <v>175</v>
+      <c r="I1" s="96" t="s">
+        <v>174</v>
       </c>
-      <c r="J1" s="97"/>
+      <c r="J1" s="98"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="128"/>
       <c r="B2" s="128"/>
       <c r="C2" s="128"/>
-      <c r="D2" s="81"/>
+      <c r="D2" s="82"/>
       <c r="E2" s="79"/>
-      <c r="F2" s="81"/>
+      <c r="F2" s="82"/>
       <c r="G2" s="79"/>
       <c r="H2" s="79"/>
       <c r="I2" s="35" t="s">
@@ -10734,30 +10731,30 @@
       </c>
       <c r="B1" s="47"/>
       <c r="C1" s="73" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D1" s="74"/>
       <c r="E1" s="75"/>
       <c r="F1" s="73" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G1" s="74"/>
       <c r="H1" s="75"/>
-      <c r="I1" s="106" t="s">
+      <c r="I1" s="103" t="s">
         <v>63</v>
       </c>
-      <c r="J1" s="108"/>
+      <c r="J1" s="105"/>
       <c r="K1" s="130" t="s">
         <v>71</v>
       </c>
       <c r="L1" s="72" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="129"/>
       <c r="B2" s="48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C2" s="72" t="s">
         <v>48</v>
@@ -10799,7 +10796,7 @@
         <v>18</v>
       </c>
       <c r="J3" s="46" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="K3" s="130"/>
       <c r="L3" s="72"/>
@@ -13650,16 +13647,16 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="50" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B2" s="54" t="s">
         <v>18</v>
       </c>
       <c r="C2" s="55" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D2" s="56" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -14897,19 +14894,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="80" t="s">
-        <v>148</v>
+      <c r="A1" s="81" t="s">
+        <v>147</v>
       </c>
       <c r="B1" s="78" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="80" t="s">
-        <v>149</v>
+      <c r="C1" s="81" t="s">
+        <v>148</v>
       </c>
-      <c r="D1" s="80" t="s">
+      <c r="D1" s="81" t="s">
         <v>72</v>
       </c>
-      <c r="E1" s="80" t="s">
+      <c r="E1" s="81" t="s">
         <v>73</v>
       </c>
       <c r="F1" s="78" t="s">
@@ -14920,11 +14917,11 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="81"/>
+      <c r="A2" s="82"/>
       <c r="B2" s="79"/>
-      <c r="C2" s="81"/>
-      <c r="D2" s="81"/>
-      <c r="E2" s="81"/>
+      <c r="C2" s="82"/>
+      <c r="D2" s="82"/>
+      <c r="E2" s="82"/>
       <c r="F2" s="79"/>
       <c r="G2" s="79"/>
     </row>
@@ -18242,11 +18239,11 @@
         <v>67</v>
       </c>
       <c r="B1" s="71" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C1" s="71"/>
       <c r="D1" s="72" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E1" s="72"/>
       <c r="F1" s="72"/>
@@ -18258,7 +18255,7 @@
       <c r="L1" s="72"/>
       <c r="M1" s="72"/>
       <c r="N1" s="71" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="O1" s="71"/>
       <c r="P1" s="71"/>
@@ -18308,40 +18305,40 @@
       <c r="B3" s="71"/>
       <c r="C3" s="71"/>
       <c r="D3" s="76" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E3" s="77"/>
       <c r="F3" s="76" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G3" s="77"/>
       <c r="H3" s="78" t="s">
         <v>48</v>
       </c>
       <c r="I3" s="76" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J3" s="77"/>
       <c r="K3" s="76" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L3" s="77"/>
       <c r="M3" s="78" t="s">
         <v>48</v>
       </c>
       <c r="N3" s="71" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O3" s="71"/>
       <c r="P3" s="71" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="Q3" s="71"/>
       <c r="R3" s="71"/>
       <c r="S3" s="71"/>
       <c r="T3" s="71"/>
       <c r="U3" s="72" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="V3" s="72"/>
       <c r="W3" s="72"/>
@@ -18350,13 +18347,13 @@
     <row r="4" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="71"/>
       <c r="B4" s="31" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C4" s="32" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="35" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E4" s="35" t="s">
         <v>4</v>
@@ -18369,7 +18366,7 @@
       </c>
       <c r="H4" s="79"/>
       <c r="I4" s="35" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J4" s="35" t="s">
         <v>4</v>
@@ -18403,16 +18400,16 @@
         <v>10</v>
       </c>
       <c r="U4" s="35" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="V4" s="35" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="W4" s="35" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="X4" s="35" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.2">
@@ -23655,44 +23652,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A1" s="83" t="s">
+      <c r="A1" s="84" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="92" t="s">
+      <c r="B1" s="93" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="93"/>
-      <c r="D1" s="93"/>
-      <c r="E1" s="93"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="95" t="s">
+      <c r="C1" s="94"/>
+      <c r="D1" s="94"/>
+      <c r="E1" s="94"/>
+      <c r="F1" s="95"/>
+      <c r="G1" s="96" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="96"/>
-      <c r="I1" s="97"/>
-      <c r="J1" s="80" t="s">
-        <v>191</v>
+      <c r="H1" s="97"/>
+      <c r="I1" s="98"/>
+      <c r="J1" s="81" t="s">
+        <v>190</v>
       </c>
-      <c r="K1" s="89" t="s">
-        <v>101</v>
+      <c r="K1" s="90" t="s">
+        <v>100</v>
       </c>
-      <c r="L1" s="92" t="s">
-        <v>90</v>
+      <c r="L1" s="93" t="s">
+        <v>89</v>
       </c>
-      <c r="M1" s="93"/>
-      <c r="N1" s="93"/>
-      <c r="O1" s="93"/>
-      <c r="P1" s="94"/>
+      <c r="M1" s="94"/>
+      <c r="N1" s="94"/>
+      <c r="O1" s="94"/>
+      <c r="P1" s="95"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A2" s="84"/>
+      <c r="A2" s="85"/>
       <c r="B2" s="71" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="98" t="s">
-        <v>95</v>
+      <c r="C2" s="99" t="s">
+        <v>94</v>
       </c>
-      <c r="D2" s="99" t="s">
+      <c r="D2" s="100" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="78" t="s">
@@ -23701,54 +23698,54 @@
       <c r="F2" s="72" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="100" t="s">
-        <v>94</v>
+      <c r="G2" s="101" t="s">
+        <v>93</v>
       </c>
-      <c r="H2" s="80" t="s">
+      <c r="H2" s="81" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="86" t="s">
-        <v>178</v>
+      <c r="I2" s="87" t="s">
+        <v>177</v>
       </c>
-      <c r="J2" s="88"/>
-      <c r="K2" s="90"/>
-      <c r="L2" s="82" t="s">
+      <c r="J2" s="89"/>
+      <c r="K2" s="91"/>
+      <c r="L2" s="83" t="s">
+        <v>163</v>
+      </c>
+      <c r="M2" s="83"/>
+      <c r="N2" s="83" t="s">
         <v>164</v>
       </c>
-      <c r="M2" s="82"/>
-      <c r="N2" s="82" t="s">
-        <v>165</v>
-      </c>
-      <c r="O2" s="82"/>
-      <c r="P2" s="101" t="s">
+      <c r="O2" s="83"/>
+      <c r="P2" s="80" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A3" s="85"/>
+      <c r="A3" s="86"/>
       <c r="B3" s="71"/>
-      <c r="C3" s="98"/>
-      <c r="D3" s="99"/>
+      <c r="C3" s="99"/>
+      <c r="D3" s="100"/>
       <c r="E3" s="79"/>
       <c r="F3" s="72"/>
-      <c r="G3" s="100"/>
-      <c r="H3" s="81"/>
-      <c r="I3" s="87"/>
-      <c r="J3" s="81"/>
-      <c r="K3" s="91"/>
+      <c r="G3" s="101"/>
+      <c r="H3" s="82"/>
+      <c r="I3" s="88"/>
+      <c r="J3" s="82"/>
+      <c r="K3" s="92"/>
       <c r="L3" s="38" t="s">
         <v>3</v>
       </c>
       <c r="M3" s="42" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N3" s="39" t="s">
         <v>3</v>
       </c>
       <c r="O3" s="42" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
-      <c r="P3" s="101"/>
+      <c r="P3" s="80"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
@@ -27353,6 +27350,7 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="qEGKRn65ciVDbmHEo86MTKkORNnkHlArZ7cMC5oUrnKH3puj0UsvJ2HCr2az9DaWSJb9lX+VmSVn49E01kPxMg==" saltValue="vQ5Ac/JH37NsP5rCz6/aCw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
+    <mergeCell ref="G2:G3"/>
     <mergeCell ref="P2:P3"/>
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="N2:O2"/>
@@ -27369,7 +27367,6 @@
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="E2:E3"/>
     <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:G3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3 C2:C3 G2:H3 O4 K1 J1:J3" xr:uid="{DA10A34B-1BA4-48EB-B541-1349E1B06C98}">
@@ -27414,18 +27411,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="83" t="s">
+      <c r="A1" s="84" t="s">
         <v>67</v>
       </c>
       <c r="B1" s="102" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C1" s="102"/>
       <c r="D1" s="102"/>
       <c r="E1" s="102"/>
       <c r="F1" s="102"/>
       <c r="G1" s="102" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H1" s="102"/>
       <c r="I1" s="102"/>
@@ -27433,9 +27430,9 @@
       <c r="K1" s="102"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="84"/>
+      <c r="A2" s="85"/>
       <c r="B2" s="73" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C2" s="74"/>
       <c r="D2" s="74"/>
@@ -27444,7 +27441,7 @@
         <v>48</v>
       </c>
       <c r="G2" s="73" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H2" s="74"/>
       <c r="I2" s="74"/>
@@ -27454,9 +27451,9 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="85"/>
+      <c r="A3" s="86"/>
       <c r="B3" s="35" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C3" s="35" t="s">
         <v>4</v>
@@ -27469,7 +27466,7 @@
       </c>
       <c r="F3" s="79"/>
       <c r="G3" s="35" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H3" s="35" t="s">
         <v>4</v>
@@ -30152,11 +30149,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="A1" s="83" t="s">
+      <c r="A1" s="84" t="s">
         <v>67</v>
       </c>
       <c r="B1" s="73" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C1" s="74"/>
       <c r="D1" s="74"/>
@@ -30177,7 +30174,7 @@
       <c r="S1" s="74"/>
       <c r="T1" s="75"/>
       <c r="U1" s="73" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="V1" s="74"/>
       <c r="W1" s="74"/>
@@ -30192,7 +30189,7 @@
       <c r="AF1" s="74"/>
       <c r="AG1" s="75"/>
       <c r="AH1" s="73" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AI1" s="74"/>
       <c r="AJ1" s="74"/>
@@ -30203,37 +30200,37 @@
       <c r="AO1" s="74"/>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="A2" s="84"/>
+      <c r="A2" s="85"/>
       <c r="B2" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="C2" s="78" t="s">
         <v>179</v>
       </c>
-      <c r="C2" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="D2" s="80" t="s">
-        <v>103</v>
+      <c r="D2" s="81" t="s">
+        <v>102</v>
       </c>
       <c r="E2" s="72" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F2" s="72"/>
       <c r="G2" s="72"/>
       <c r="H2" s="72" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I2" s="72"/>
       <c r="J2" s="72"/>
       <c r="K2" s="78" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="L2" s="73" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="M2" s="74"/>
       <c r="N2" s="74"/>
       <c r="O2" s="75"/>
       <c r="P2" s="73" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="Q2" s="74"/>
       <c r="R2" s="75"/>
@@ -30242,7 +30239,7 @@
       </c>
       <c r="T2" s="75"/>
       <c r="U2" s="72" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="V2" s="72" t="s">
         <v>22</v>
@@ -30280,28 +30277,28 @@
       <c r="AG2" s="72" t="s">
         <v>32</v>
       </c>
-      <c r="AH2" s="95" t="s">
+      <c r="AH2" s="96" t="s">
+        <v>120</v>
+      </c>
+      <c r="AI2" s="98"/>
+      <c r="AJ2" s="96" t="s">
         <v>121</v>
       </c>
-      <c r="AI2" s="97"/>
-      <c r="AJ2" s="95" t="s">
+      <c r="AK2" s="98"/>
+      <c r="AL2" s="96" t="s">
         <v>122</v>
       </c>
-      <c r="AK2" s="97"/>
-      <c r="AL2" s="95" t="s">
+      <c r="AM2" s="98"/>
+      <c r="AN2" s="96" t="s">
         <v>123</v>
       </c>
-      <c r="AM2" s="97"/>
-      <c r="AN2" s="95" t="s">
-        <v>124</v>
-      </c>
-      <c r="AO2" s="97"/>
+      <c r="AO2" s="98"/>
     </row>
     <row r="3" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="A3" s="85"/>
+      <c r="A3" s="86"/>
       <c r="B3" s="79"/>
       <c r="C3" s="79"/>
-      <c r="D3" s="81"/>
+      <c r="D3" s="82"/>
       <c r="E3" s="43" t="s">
         <v>19</v>
       </c>
@@ -30309,7 +30306,7 @@
         <v>20</v>
       </c>
       <c r="G3" s="44" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H3" s="43" t="s">
         <v>19</v>
@@ -30318,35 +30315,35 @@
         <v>20</v>
       </c>
       <c r="J3" s="44" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K3" s="79"/>
       <c r="L3" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="M3" s="35" t="s">
         <v>105</v>
       </c>
-      <c r="M3" s="35" t="s">
+      <c r="N3" s="35" t="s">
         <v>106</v>
       </c>
-      <c r="N3" s="35" t="s">
+      <c r="O3" s="35" t="s">
         <v>107</v>
       </c>
-      <c r="O3" s="35" t="s">
+      <c r="P3" s="35" t="s">
         <v>108</v>
       </c>
-      <c r="P3" s="35" t="s">
+      <c r="Q3" s="35" t="s">
         <v>109</v>
       </c>
-      <c r="Q3" s="35" t="s">
+      <c r="R3" s="35" t="s">
         <v>110</v>
-      </c>
-      <c r="R3" s="35" t="s">
-        <v>111</v>
       </c>
       <c r="S3" s="32" t="s">
         <v>18</v>
       </c>
       <c r="T3" s="46" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="U3" s="72"/>
       <c r="V3" s="72"/>
@@ -30362,28 +30359,28 @@
       <c r="AF3" s="72"/>
       <c r="AG3" s="72"/>
       <c r="AH3" s="45" t="s">
+        <v>111</v>
+      </c>
+      <c r="AI3" s="36" t="s">
         <v>112</v>
       </c>
-      <c r="AI3" s="36" t="s">
-        <v>113</v>
+      <c r="AJ3" s="36" t="s">
+        <v>114</v>
       </c>
-      <c r="AJ3" s="36" t="s">
+      <c r="AK3" s="36" t="s">
         <v>115</v>
       </c>
-      <c r="AK3" s="36" t="s">
+      <c r="AL3" s="36" t="s">
         <v>116</v>
       </c>
-      <c r="AL3" s="36" t="s">
+      <c r="AM3" s="36" t="s">
         <v>117</v>
       </c>
-      <c r="AM3" s="36" t="s">
+      <c r="AN3" s="36" t="s">
         <v>118</v>
       </c>
-      <c r="AN3" s="36" t="s">
+      <c r="AO3" s="36" t="s">
         <v>119</v>
-      </c>
-      <c r="AO3" s="36" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:41" x14ac:dyDescent="0.2">
@@ -38989,6 +38986,20 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="in9HWhrbfPeQLKOphe9HcQ3ZWSvu9v4Chn7tSlbMDS+5w+WrRSh6fFRY7HaRetWtqRaeTChN5KnyLnOrPZ3pZA==" saltValue="7WB/oWTeA55ZXeyLP0lXUw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="30">
+    <mergeCell ref="AD2:AD3"/>
+    <mergeCell ref="AE2:AE3"/>
+    <mergeCell ref="AF2:AF3"/>
+    <mergeCell ref="AG2:AG3"/>
+    <mergeCell ref="W2:W3"/>
+    <mergeCell ref="X2:X3"/>
+    <mergeCell ref="Y2:Y3"/>
+    <mergeCell ref="Z2:Z3"/>
+    <mergeCell ref="AA2:AA3"/>
+    <mergeCell ref="S2:T2"/>
+    <mergeCell ref="U2:U3"/>
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="AB2:AB3"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="AN2:AO2"/>
@@ -39005,20 +39016,6 @@
     <mergeCell ref="AC2:AC3"/>
     <mergeCell ref="L2:O2"/>
     <mergeCell ref="P2:R2"/>
-    <mergeCell ref="S2:T2"/>
-    <mergeCell ref="U2:U3"/>
-    <mergeCell ref="V2:V3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="AB2:AB3"/>
-    <mergeCell ref="AD2:AD3"/>
-    <mergeCell ref="AE2:AE3"/>
-    <mergeCell ref="AF2:AF3"/>
-    <mergeCell ref="AG2:AG3"/>
-    <mergeCell ref="W2:W3"/>
-    <mergeCell ref="X2:X3"/>
-    <mergeCell ref="Y2:Y3"/>
-    <mergeCell ref="Z2:Z3"/>
-    <mergeCell ref="AA2:AA3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D3 L3:R3 AH3:AO3" xr:uid="{259DA634-7C5F-4453-A9E2-D13FC35BABDC}">
@@ -39068,36 +39065,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="85" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="85" t="s">
+      <c r="B1" s="86" t="s">
+        <v>170</v>
+      </c>
+      <c r="C1" s="86"/>
+      <c r="D1" s="93" t="s">
         <v>171</v>
       </c>
-      <c r="C1" s="85"/>
-      <c r="D1" s="92" t="s">
+      <c r="E1" s="94"/>
+      <c r="F1" s="94"/>
+      <c r="G1" s="94"/>
+      <c r="H1" s="94"/>
+      <c r="I1" s="94"/>
+      <c r="J1" s="95"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" s="85"/>
+      <c r="B2" s="84" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="84" t="s">
+        <v>181</v>
+      </c>
+      <c r="D2" s="84" t="s">
         <v>172</v>
       </c>
-      <c r="E1" s="93"/>
-      <c r="F1" s="93"/>
-      <c r="G1" s="93"/>
-      <c r="H1" s="93"/>
-      <c r="I1" s="93"/>
-      <c r="J1" s="94"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="84"/>
-      <c r="B2" s="83" t="s">
-        <v>58</v>
-      </c>
-      <c r="C2" s="83" t="s">
-        <v>182</v>
-      </c>
-      <c r="D2" s="83" t="s">
-        <v>173</v>
-      </c>
       <c r="E2" s="73" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F2" s="75"/>
       <c r="G2" s="73" t="s">
@@ -39108,12 +39105,12 @@
       <c r="J2" s="75"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="85"/>
-      <c r="B3" s="85"/>
-      <c r="C3" s="85"/>
-      <c r="D3" s="85"/>
+      <c r="A3" s="86"/>
+      <c r="B3" s="86"/>
+      <c r="C3" s="86"/>
+      <c r="D3" s="86"/>
       <c r="E3" s="35" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F3" s="44" t="s">
         <v>49</v>
@@ -39122,13 +39119,13 @@
         <v>54</v>
       </c>
       <c r="H3" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="I3" s="35" t="s">
         <v>110</v>
       </c>
-      <c r="I3" s="35" t="s">
-        <v>111</v>
-      </c>
       <c r="J3" s="35" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
@@ -41587,127 +41584,127 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A1" s="83" t="s">
+      <c r="A1" s="84" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="83" t="s">
-        <v>91</v>
+      <c r="B1" s="84" t="s">
+        <v>90</v>
       </c>
-      <c r="C1" s="103" t="s">
+      <c r="C1" s="116" t="s">
+        <v>130</v>
+      </c>
+      <c r="D1" s="118"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="31" t="s">
         <v>131</v>
       </c>
-      <c r="D1" s="105"/>
-      <c r="E1" s="104"/>
-      <c r="F1" s="31" t="s">
+      <c r="G1" s="103" t="s">
         <v>132</v>
       </c>
-      <c r="G1" s="106" t="s">
+      <c r="H1" s="104"/>
+      <c r="I1" s="105"/>
+      <c r="J1" s="110" t="s">
         <v>133</v>
       </c>
-      <c r="H1" s="107"/>
-      <c r="I1" s="108"/>
-      <c r="J1" s="113" t="s">
-        <v>134</v>
-      </c>
-      <c r="K1" s="114"/>
-      <c r="L1" s="114"/>
-      <c r="M1" s="115"/>
+      <c r="K1" s="111"/>
+      <c r="L1" s="111"/>
+      <c r="M1" s="112"/>
       <c r="N1" s="71" t="s">
         <v>61</v>
       </c>
-      <c r="O1" s="106" t="s">
+      <c r="O1" s="103" t="s">
         <v>62</v>
       </c>
-      <c r="P1" s="107"/>
-      <c r="Q1" s="107"/>
-      <c r="R1" s="107"/>
-      <c r="S1" s="108"/>
+      <c r="P1" s="104"/>
+      <c r="Q1" s="104"/>
+      <c r="R1" s="104"/>
+      <c r="S1" s="105"/>
       <c r="T1" s="72" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
-      <c r="U1" s="110" t="s">
+      <c r="U1" s="107" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A2" s="84"/>
-      <c r="B2" s="84"/>
-      <c r="C2" s="83" t="s">
+      <c r="A2" s="85"/>
+      <c r="B2" s="85"/>
+      <c r="C2" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="D2" s="103" t="s">
+      <c r="D2" s="116" t="s">
         <v>47</v>
       </c>
-      <c r="E2" s="104"/>
-      <c r="F2" s="83" t="s">
+      <c r="E2" s="117"/>
+      <c r="F2" s="84" t="s">
         <v>48</v>
       </c>
       <c r="G2" s="76"/>
-      <c r="H2" s="109"/>
+      <c r="H2" s="106"/>
       <c r="I2" s="77"/>
-      <c r="J2" s="116"/>
-      <c r="K2" s="117"/>
-      <c r="L2" s="117"/>
-      <c r="M2" s="118"/>
+      <c r="J2" s="113"/>
+      <c r="K2" s="114"/>
+      <c r="L2" s="114"/>
+      <c r="M2" s="115"/>
       <c r="N2" s="71"/>
       <c r="O2" s="76"/>
-      <c r="P2" s="109"/>
-      <c r="Q2" s="109"/>
-      <c r="R2" s="109"/>
+      <c r="P2" s="106"/>
+      <c r="Q2" s="106"/>
+      <c r="R2" s="106"/>
       <c r="S2" s="77"/>
       <c r="T2" s="72"/>
-      <c r="U2" s="111"/>
+      <c r="U2" s="108"/>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A3" s="85"/>
-      <c r="B3" s="85"/>
-      <c r="C3" s="85"/>
+      <c r="A3" s="86"/>
+      <c r="B3" s="86"/>
+      <c r="C3" s="86"/>
       <c r="D3" s="33" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="85"/>
+      <c r="F3" s="86"/>
       <c r="G3" s="35" t="s">
+        <v>134</v>
+      </c>
+      <c r="H3" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="H3" s="35" t="s">
+      <c r="I3" s="35" t="s">
         <v>136</v>
       </c>
-      <c r="I3" s="35" t="s">
+      <c r="J3" s="41" t="s">
+        <v>99</v>
+      </c>
+      <c r="K3" s="41" t="s">
         <v>137</v>
       </c>
-      <c r="J3" s="41" t="s">
-        <v>100</v>
-      </c>
-      <c r="K3" s="41" t="s">
+      <c r="L3" s="41" t="s">
         <v>138</v>
       </c>
-      <c r="L3" s="41" t="s">
+      <c r="M3" s="41" t="s">
         <v>139</v>
-      </c>
-      <c r="M3" s="41" t="s">
-        <v>140</v>
       </c>
       <c r="N3" s="71"/>
       <c r="O3" s="34" t="s">
         <v>60</v>
       </c>
       <c r="P3" s="57" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="Q3" s="35" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="R3" s="35" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="S3" s="32" t="s">
         <v>34</v>
       </c>
       <c r="T3" s="72"/>
-      <c r="U3" s="112"/>
+      <c r="U3" s="109"/>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
@@ -46313,18 +46310,18 @@
   <sheetProtection algorithmName="SHA-512" hashValue="vb3l2GPyTmOeMpvedAjZ5so+j03iBDjWx3ozUq1oM5QjY9AJ+7qSyqXmIAxigMK0wo/0kW2bwbQpgi37D24U6w==" saltValue="804oboBvFb3X5NzoXiRygQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <dataConsolidate/>
   <mergeCells count="12">
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="G1:I2"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
     <mergeCell ref="O1:S2"/>
     <mergeCell ref="U1:U3"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="J1:M2"/>
     <mergeCell ref="N1:N3"/>
     <mergeCell ref="T1:T3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="G1:I2"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" sqref="U1:U3 Q3:R3 G3:M3" xr:uid="{AF5AE5B6-046A-4AF7-91CF-4FE32EB3CEA6}">
@@ -46365,47 +46362,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="83" t="s">
+      <c r="A1" s="84" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="89" t="s">
-        <v>142</v>
+      <c r="B1" s="90" t="s">
+        <v>141</v>
       </c>
       <c r="C1" s="119" t="s">
         <v>64</v>
       </c>
       <c r="D1" s="120"/>
-      <c r="E1" s="89" t="s">
+      <c r="E1" s="90" t="s">
+        <v>142</v>
+      </c>
+      <c r="F1" s="84" t="s">
         <v>143</v>
       </c>
-      <c r="F1" s="83" t="s">
-        <v>144</v>
-      </c>
-      <c r="G1" s="113" t="s">
+      <c r="G1" s="110" t="s">
         <v>34</v>
       </c>
-      <c r="H1" s="114"/>
-      <c r="I1" s="115"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="112"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="85"/>
-      <c r="B2" s="91"/>
+      <c r="A2" s="86"/>
+      <c r="B2" s="92"/>
       <c r="C2" s="41" t="s">
         <v>54</v>
       </c>
       <c r="D2" s="41" t="s">
         <v>65</v>
       </c>
-      <c r="E2" s="91"/>
-      <c r="F2" s="85"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="86"/>
       <c r="G2" s="51" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H2" s="31" t="s">
         <v>35</v>
       </c>
       <c r="I2" s="41" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -48659,42 +48656,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1" s="83" t="s">
+      <c r="A1" s="84" t="s">
         <v>67</v>
       </c>
       <c r="B1" s="78" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C1" s="78" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D1" s="123" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E1" s="125" t="s">
         <v>64</v>
       </c>
       <c r="F1" s="126"/>
-      <c r="G1" s="80" t="s">
-        <v>143</v>
+      <c r="G1" s="81" t="s">
+        <v>142</v>
       </c>
       <c r="H1" s="121" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I1" s="73" t="s">
         <v>34</v>
       </c>
       <c r="J1" s="75"/>
-      <c r="K1" s="80" t="s">
-        <v>145</v>
+      <c r="K1" s="81" t="s">
+        <v>144</v>
       </c>
       <c r="L1" s="73" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="M1" s="75"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="85"/>
+      <c r="A2" s="86"/>
       <c r="B2" s="79"/>
       <c r="C2" s="79"/>
       <c r="D2" s="124"/>
@@ -48704,20 +48701,20 @@
       <c r="F2" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="G2" s="81"/>
+      <c r="G2" s="82"/>
       <c r="H2" s="122"/>
       <c r="I2" s="53" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J2" s="52" t="s">
         <v>35</v>
       </c>
-      <c r="K2" s="81"/>
+      <c r="K2" s="82"/>
       <c r="L2" s="35" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M2" s="35" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">

</xml_diff>